<commit_message>
feat: add social media data collection, preprocessing pipelines, and sentiment analysis scripts
</commit_message>
<xml_diff>
--- a/data/evaluasi_komparasi_sentimen.xlsx
+++ b/data/evaluasi_komparasi_sentimen.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan Perbandingan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metrik Per Kelas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Confusion Matrices" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ringkasan Perbandingan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Metrik Per Kelas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Confusion Matrices" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +36,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -47,21 +44,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,41 +415,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Paradigma</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Metode</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Akurasi</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Precision (Macro)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Recall (Macro)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>F1-Score (Macro)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>F1-Score (Weighted)</t>
         </is>
@@ -480,212 +468,175 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>99.19%</t>
+          <t>83.90%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>98.67%</t>
+          <t>67.15%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>98.41%</t>
+          <t>68.18%</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>98.51%</t>
+          <t>67.64%</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>99.19%</t>
+          <t>84.09%</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Distance Metric</t>
+          <t>Machine Learning (Baseline)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cosine Similarity</t>
+          <t>Linear SVM</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>67.74%</t>
+          <t>75.12%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>58.03%</t>
+          <t>51.62%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>59.67%</t>
+          <t>51.37%</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>58.73%</t>
+          <t>51.49%</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>68.39%</t>
+          <t>74.99%</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Machine Learning (Baseline)</t>
+          <t>Machine Learning (Hybrid)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Linear SVM</t>
+          <t>Hybrid SVM (TF-IDF + InSet)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>70.16%</t>
+          <t>76.59%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>64.66%</t>
+          <t>56.97%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>49.50%</t>
+          <t>57.56%</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>51.74%</t>
+          <t>57.13%</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>65.74%</t>
+          <t>77.08%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Machine Learning (Hybrid)</t>
+          <t>Distance Metric</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hybrid SVM (TF-IDF + InSet)</t>
+          <t>Cosine Similarity</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>92.74%</t>
+          <t>67.32%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>90.15%</t>
+          <t>44.64%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>87.30%</t>
+          <t>50.53%</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>87.71%</t>
+          <t>46.18%</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>92.36%</t>
+          <t>70.14%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Deep Learning</t>
+          <t>X-Shot Learning</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Neural BiLSTM (Attention)</t>
+          <t>X-Shot Reasoning (CoT)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>64.52%</t>
+          <t>24.39%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>58.42%</t>
+          <t>44.43%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>63.78%</t>
+          <t>38.20%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>58.58%</t>
+          <t>20.36%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>66.48%</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>X-Shot Learning</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>X-Shot Reasoning (CoT)</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>44.35%</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>73.98%</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>48.94%</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>39.40%</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>45.88%</t>
+          <t>25.65%</t>
         </is>
       </c>
     </row>
@@ -700,36 +651,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metode</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Kelas Sentimen</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Precision</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Recall</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>F1-Score</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Support</t>
         </is>
@@ -748,21 +699,21 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>91.46%</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>90.36%</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>90.91%</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>79</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3">
@@ -778,17 +729,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>96.00%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>54.17%</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>97.96%</t>
+          <t>52.00%</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -808,27 +759,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>95.24%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>97.56%</t>
+          <t>60.00%</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cosine Similarity</t>
+          <t>Linear SVM</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -838,27 +789,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>82.43%</t>
+          <t>84.43%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>77.22%</t>
+          <t>84.94%</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>79.74%</t>
+          <t>84.68%</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>79</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cosine Similarity</t>
+          <t>Linear SVM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -868,17 +819,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>30.43%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>54.17%</t>
+          <t>29.17%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>52.00%</t>
+          <t>29.79%</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -888,7 +839,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cosine Similarity</t>
+          <t>Linear SVM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -898,27 +849,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>41.67%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>47.62%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>44.44%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Linear SVM</t>
+          <t>Hybrid SVM (TF-IDF + InSet)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -928,27 +879,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>72.82%</t>
+          <t>86.42%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>94.94%</t>
+          <t>84.34%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>82.42%</t>
+          <t>85.37%</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>79</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Linear SVM</t>
+          <t>Hybrid SVM (TF-IDF + InSet)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -958,17 +909,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>75.00%</t>
+          <t>34.48%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>25.00%</t>
+          <t>41.67%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>37.50%</t>
+          <t>37.74%</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -978,7 +929,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Linear SVM</t>
+          <t>Hybrid SVM (TF-IDF + InSet)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -988,27 +939,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>46.15%</t>
+          <t>50.00%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>28.57%</t>
+          <t>46.67%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>35.29%</t>
+          <t>48.28%</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hybrid SVM</t>
+          <t>Cosine Similarity</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1018,27 +969,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>96.34%</t>
+          <t>86.01%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>100.00%</t>
+          <t>74.10%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>98.14%</t>
+          <t>79.61%</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>79</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hybrid SVM</t>
+          <t>Cosine Similarity</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1048,17 +999,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>94.12%</t>
+          <t>26.47%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>66.67%</t>
+          <t>37.50%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>78.05%</t>
+          <t>31.03%</t>
         </is>
       </c>
       <c r="F12" t="n">
@@ -1068,7 +1019,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hybrid SVM</t>
+          <t>Cosine Similarity</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1078,27 +1029,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>80.00%</t>
+          <t>21.43%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>95.24%</t>
+          <t>40.00%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>86.96%</t>
+          <t>27.91%</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Neural BiLSTM</t>
+          <t>X-Shot Reasoning</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1108,27 +1059,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>91.07%</t>
+          <t>87.10%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>64.56%</t>
+          <t>16.27%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>75.56%</t>
+          <t>27.41%</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>79</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Neural BiLSTM</t>
+          <t>X-Shot Reasoning</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1138,17 +1089,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>44.19%</t>
+          <t>12.87%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>79.17%</t>
+          <t>91.67%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>56.72%</t>
+          <t>22.56%</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1158,7 +1109,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Neural BiLSTM</t>
+          <t>X-Shot Reasoning</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1168,111 +1119,21 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>40.00%</t>
+          <t>33.33%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>47.62%</t>
+          <t>6.67%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>43.48%</t>
+          <t>11.11%</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>X-Shot Reasoning</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Negatif</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>96.67%</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>36.71%</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>53.21%</t>
-        </is>
-      </c>
-      <c r="F17" t="n">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>X-Shot Reasoning</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Netral</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>25.27%</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>95.83%</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>40.00%</t>
-        </is>
-      </c>
-      <c r="F18" t="n">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>X-Shot Reasoning</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Positif</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>100.00%</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>14.29%</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>25.00%</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1286,31 +1147,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metode</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Aktual (Ground Truth)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Prediksi: Negatif</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Prediksi: Netral</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Prediksi: Positif</t>
         </is>
@@ -1328,13 +1189,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>79</v>
+        <v>150</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -1349,13 +1210,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="D3" t="n">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -1370,19 +1231,19 @@
         </is>
       </c>
       <c r="C4" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cosine Similarity</t>
+          <t>Linear SVM</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1391,19 +1252,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>61</v>
+        <v>141</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cosine Similarity</t>
+          <t>Linear SVM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1412,19 +1273,19 @@
         </is>
       </c>
       <c r="C6" t="n">
+        <v>17</v>
+      </c>
+      <c r="D6" t="n">
         <v>7</v>
       </c>
-      <c r="D6" t="n">
-        <v>13</v>
-      </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cosine Similarity</t>
+          <t>Linear SVM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1433,19 +1294,19 @@
         </is>
       </c>
       <c r="C7" t="n">
+        <v>9</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>6</v>
-      </c>
-      <c r="D7" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Linear SVM</t>
+          <t>Hybrid SVM (TF-IDF + InSet)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1454,19 +1315,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>75</v>
+        <v>140</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="E8" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Linear SVM</t>
+          <t>Hybrid SVM (TF-IDF + InSet)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1475,19 +1336,19 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Linear SVM</t>
+          <t>Hybrid SVM (TF-IDF + InSet)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1496,19 +1357,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hybrid SVM</t>
+          <t>Cosine Similarity</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1517,19 +1378,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>79</v>
+        <v>123</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hybrid SVM</t>
+          <t>Cosine Similarity</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1538,19 +1399,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D12" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E12" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hybrid SVM</t>
+          <t>Cosine Similarity</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1559,19 +1420,19 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Neural BiLSTM</t>
+          <t>X-Shot Reasoning</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1580,19 +1441,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="D14" t="n">
-        <v>16</v>
+        <v>137</v>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Neural BiLSTM</t>
+          <t>X-Shot Reasoning</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1604,16 +1465,16 @@
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Neural BiLSTM</t>
+          <t>X-Shot Reasoning</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1622,76 +1483,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>X-Shot Reasoning</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Negatif</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>29</v>
-      </c>
-      <c r="D17" t="n">
-        <v>50</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>X-Shot Reasoning</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Netral</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
         <v>1</v>
-      </c>
-      <c r="D18" t="n">
-        <v>23</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>X-Shot Reasoning</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Positif</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>18</v>
-      </c>
-      <c r="E19" t="n">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: selaraskan analisis sentimen ke krisis kelangkaan BBM & hapus artefak ketenagakerjaan
</commit_message>
<xml_diff>
--- a/data/evaluasi_komparasi_sentimen.xlsx
+++ b/data/evaluasi_komparasi_sentimen.xlsx
@@ -616,27 +616,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>24.39%</t>
+          <t>29.76%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>44.43%</t>
+          <t>40.78%</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>38.20%</t>
+          <t>42.78%</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>20.36%</t>
+          <t>23.41%</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>25.65%</t>
+          <t>32.29%</t>
         </is>
       </c>
     </row>
@@ -1059,17 +1059,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>87.10%</t>
+          <t>94.74%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>16.27%</t>
+          <t>21.69%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>27.41%</t>
+          <t>35.29%</t>
         </is>
       </c>
       <c r="F14" t="n">
@@ -1089,17 +1089,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>12.87%</t>
+          <t>15.09%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>91.67%</t>
+          <t>100.00%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>22.56%</t>
+          <t>26.23%</t>
         </is>
       </c>
       <c r="F15" t="n">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>12.50%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>11.11%</t>
+          <t>8.70%</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -1441,13 +1441,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D14" t="n">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -1462,10 +1462,10 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>

</xml_diff>